<commit_message>
Add SOH report for 2026-10-08
</commit_message>
<xml_diff>
--- a/reports/SOH_07_10_2026.xlsx
+++ b/reports/SOH_07_10_2026.xlsx
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>21000</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>270</v>
+        <v>252</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1129</v>
+        <v>1148</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>40000</v>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="D32" s="2" t="n">
-        <v>813</v>
+        <v>824</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>10500</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>40000</v>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>10500</v>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="D36" s="2" t="n">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>10500</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1525,7 +1525,7 @@
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E39" s="3" t="n">
         <v>10500</v>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E40" s="3" t="n">
         <v>21000</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>51000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>167</v>
+        <v>194</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="D92" s="2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E92" s="3" t="n">
         <v>8000</v>
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="E93" s="3" t="n">
         <v>8000</v>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="E102" s="3" t="n">
         <v>4708</v>
@@ -3317,7 +3317,7 @@
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E103" s="3" t="n">
         <v>4708</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E105" s="3" t="n">
         <v>4708</v>
@@ -3541,7 +3541,7 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="E111" s="3" t="n">
         <v>25000</v>
@@ -3569,7 +3569,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="E112" s="3" t="n">
         <v>25000</v>
@@ -3625,7 +3625,7 @@
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="E114" s="3" t="n">
         <v>36000</v>
@@ -3709,7 +3709,7 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E117" s="3" t="n">
         <v>5000</v>
@@ -3737,7 +3737,7 @@
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="E118" s="3" t="n">
         <v>5000</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2207</v>
+        <v>2228</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E127" s="3" t="n">
         <v>2500</v>
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>-1</v>
+        <v>11</v>
       </c>
       <c r="E129" s="3" t="n">
         <v>2500</v>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="D174" s="2" t="n">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E174" s="3" t="n">
         <v>13500</v>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -9682,7 +9682,7 @@
         </is>
       </c>
       <c r="D334" s="2" t="n">
-        <v>537</v>
+        <v>57</v>
       </c>
       <c r="E334" s="3" t="n">
         <v>2500</v>
@@ -12804,24 +12804,24 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>5061031650942</t>
+          <t>5060677903931</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>65093</t>
+          <t>90393</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS AIR FRESHENER SCEN</t>
+          <t>CHUPA CHUPS FRESHENER CHERRY</t>
         </is>
       </c>
       <c r="D446" s="2" t="n">
-        <v>119</v>
+        <v>3</v>
       </c>
       <c r="E446" s="3" t="n">
-        <v>8220</v>
+        <v>8856</v>
       </c>
       <c r="F446" t="inlineStr">
         <is>
@@ -12832,24 +12832,24 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>5060677903931</t>
+          <t>5060677903962</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>90393</t>
+          <t>90396</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS FRESHENER CHERRY</t>
+          <t>CHUPA CHUPS FRESHENER STRAWBER</t>
         </is>
       </c>
       <c r="D447" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E447" s="3" t="n">
-        <v>8856</v>
+        <v>8855.5</v>
       </c>
       <c r="F447" t="inlineStr">
         <is>
@@ -12916,24 +12916,24 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>5060677903962</t>
+          <t>5061031650942</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>90396</t>
+          <t>65093</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>CHUPA CHUPS FRESHENER STRAWBER</t>
+          <t>CHUPA CHUPS AIR FRESHENER SCEN</t>
         </is>
       </c>
       <c r="D450" s="2" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="E450" s="3" t="n">
-        <v>8855.5</v>
+        <v>8220</v>
       </c>
       <c r="F450" t="inlineStr">
         <is>
@@ -15254,7 +15254,7 @@
         </is>
       </c>
       <c r="D533" s="2" t="n">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E533" s="3" t="n">
         <v>69124</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>4327</v>
+        <v>4231</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>10251</v>
@@ -19343,7 +19343,7 @@
         </is>
       </c>
       <c r="D679" s="2" t="n">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="E679" s="3" t="n">
         <v>2338</v>
@@ -19427,7 +19427,7 @@
         </is>
       </c>
       <c r="D682" s="2" t="n">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="E682" s="3" t="n">
         <v>6039</v>
@@ -29597,7 +29597,7 @@
         </is>
       </c>
       <c r="D1045" s="2" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E1045" s="3" t="n">
         <v>11977</v>
@@ -38389,7 +38389,7 @@
         </is>
       </c>
       <c r="D1359" s="2" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E1359" s="3" t="n">
         <v>15766</v>
@@ -39355,24 +39355,24 @@
     <row r="1394">
       <c r="A1394" t="inlineStr">
         <is>
-          <t>9333527302984</t>
+          <t>9333527379658</t>
         </is>
       </c>
       <c r="B1394" t="inlineStr">
         <is>
-          <t>OX0633</t>
+          <t>KA0368</t>
         </is>
       </c>
       <c r="C1394" t="inlineStr">
         <is>
-          <t>SOLAR STAKE ST.STEEL 36cm</t>
+          <t>SPAGHETTI SERVER NON-STICK</t>
         </is>
       </c>
       <c r="D1394" s="2" t="n">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="E1394" s="3" t="n">
-        <v>16437</v>
+        <v>11698</v>
       </c>
       <c r="F1394" t="inlineStr">
         <is>
@@ -39383,24 +39383,24 @@
     <row r="1395">
       <c r="A1395" t="inlineStr">
         <is>
-          <t>9333527379627</t>
+          <t>9333527379634</t>
         </is>
       </c>
       <c r="B1395" t="inlineStr">
         <is>
-          <t>KA0365</t>
+          <t>KA0366</t>
         </is>
       </c>
       <c r="C1395" t="inlineStr">
         <is>
-          <t>SOUP LADLE NON-STICK</t>
+          <t>SPATULA NON-STICK</t>
         </is>
       </c>
       <c r="D1395" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E1395" s="3" t="n">
-        <v>11698</v>
+        <v>15124</v>
       </c>
       <c r="F1395" t="inlineStr">
         <is>
@@ -39411,17 +39411,17 @@
     <row r="1396">
       <c r="A1396" t="inlineStr">
         <is>
-          <t>9333527379658</t>
+          <t>9333527379627</t>
         </is>
       </c>
       <c r="B1396" t="inlineStr">
         <is>
-          <t>KA0368</t>
+          <t>KA0365</t>
         </is>
       </c>
       <c r="C1396" t="inlineStr">
         <is>
-          <t>SPAGHETTI SERVER NON-STICK</t>
+          <t>SOUP LADLE NON-STICK</t>
         </is>
       </c>
       <c r="D1396" s="2" t="n">
@@ -39439,24 +39439,24 @@
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
-          <t>9333527379634</t>
+          <t>9333527614131</t>
         </is>
       </c>
       <c r="B1397" t="inlineStr">
         <is>
-          <t>KA0366</t>
+          <t>PA4043</t>
         </is>
       </c>
       <c r="C1397" t="inlineStr">
         <is>
-          <t>SPATULA NON-STICK</t>
+          <t>SPIKEY BALL SQUEAK PET TOY 3AS</t>
         </is>
       </c>
       <c r="D1397" s="2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E1397" s="3" t="n">
-        <v>15124</v>
+        <v>5118</v>
       </c>
       <c r="F1397" t="inlineStr">
         <is>
@@ -39467,24 +39467,24 @@
     <row r="1398">
       <c r="A1398" t="inlineStr">
         <is>
-          <t>9333527614131</t>
+          <t>9333527302984</t>
         </is>
       </c>
       <c r="B1398" t="inlineStr">
         <is>
-          <t>PA4043</t>
+          <t>OX0633</t>
         </is>
       </c>
       <c r="C1398" t="inlineStr">
         <is>
-          <t>SPIKEY BALL SQUEAK PET TOY 3AS</t>
+          <t>SOLAR STAKE ST.STEEL 36cm</t>
         </is>
       </c>
       <c r="D1398" s="2" t="n">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="E1398" s="3" t="n">
-        <v>5118</v>
+        <v>16437</v>
       </c>
       <c r="F1398" t="inlineStr">
         <is>
@@ -42589,7 +42589,7 @@
         </is>
       </c>
       <c r="D1509" s="2" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E1509" s="3" t="n">
         <v>41300</v>

</xml_diff>